<commit_message>
security: dependency, injection and dead-code hardening
- Replace abandoned 'xlsx' (unpatched prototype pollution + ReDoS on
  malicious files) with ExcelJS via lib/sheet.ts; own RFC-4180 CSV parser;
  prototype-less row objects; .xls no longer accepted
- Patch lodash and react-router (high); pin patched uuid; npm audit: 0
- lib/safe.ts: safeUrl (blocks javascript:/data: links), escapeHtml,
  formula-injection-safe CSV (all 5 exports; Employees export was
  unquoted and broke on commas)
- Escape printed document titles
- Intake template: header comments replaced by input messages (ExcelJS)
- Remove 168KB unused mock data and 13 unused/unsafe Supabase helpers
</commit_message>
<xml_diff>
--- a/app/public/templates/Talent_Intake_Template.xlsx
+++ b/app/public/templates/Talent_Intake_Template.xlsx
@@ -193,51 +193,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Magaya ELMS</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Pick from the list: Graduate Trainee or Attachment Student.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Recommended. Used to spot people already in ELMS.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Pick from the list.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>University or college.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>Degree or programme name.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Students only: 1 to 6.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Pick from the list, or leave blank if not decided.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7271,23 +7226,25 @@
       <c r="K501" s="8" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Programme" error="Choose Graduate Trainee or Attachment Student." type="list">
+  <dataValidations count="7">
+    <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Programme" error="Choose Graduate Trainee or Attachment Student." promptTitle="Programme *" prompt="Pick from the list: Graduate Trainee or Attachment Student." type="list">
       <formula1>=Lists!$A$2:$A$3</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gender" error="Choose from the list." type="list">
+    <dataValidation sqref="F2:F501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Gender" error="Choose from the list." promptTitle="Gender" prompt="Pick from the list." type="list">
       <formula1>=Lists!$B$2:$B$3</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Site" error="Choose a site from the list, or leave blank." type="list">
+    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Site" error="Choose a site from the list, or leave blank." promptTitle="Intended Site" prompt="Pick from the list, or leave blank if not decided." type="list">
       <formula1>=Lists!$C$2:$C$18</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Year of study" error="Enter a whole number from 1 to 6." type="whole" operator="between">
+    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Year of study" error="Enter a whole number from 1 to 6." promptTitle="Year of Study" prompt="Students only: 1 to 6." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>6</formula2>
     </dataValidation>
+    <dataValidation sqref="D2:D501" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Email" prompt="Recommended. Used to spot people already in ELMS."/>
+    <dataValidation sqref="G2:G501" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Institution" prompt="University or college."/>
+    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Field of Study" prompt="Degree or programme name."/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>